<commit_message>
Updated optimal capital structure database
</commit_message>
<xml_diff>
--- a/research/traditional_assets/database/data/anguilla/anguilla_investments_asset_management.xlsx
+++ b/research/traditional_assets/database/data/anguilla/anguilla_investments_asset_management.xlsx
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="K2">
-        <v>0.182</v>
+        <v>-0.105</v>
       </c>
       <c r="M2">
         <v>0</v>
@@ -597,7 +597,7 @@
         <v>0</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -606,58 +606,64 @@
         <v>0</v>
       </c>
       <c r="R2">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="S2">
         <v>0</v>
       </c>
       <c r="U2">
-        <v>0</v>
+        <v>0.105</v>
       </c>
       <c r="V2">
-        <v>0</v>
+        <v>0.1029411764705882</v>
       </c>
       <c r="W2">
-        <v>-0.175</v>
+        <v>0.1436388508891929</v>
       </c>
       <c r="X2">
-        <v>0.1427779612909701</v>
+        <v>0.1647033579267986</v>
       </c>
       <c r="Y2">
-        <v>-0.3177779612909701</v>
+        <v>-0.02106450703760576</v>
       </c>
       <c r="AB2">
-        <v>0.1391722223025425</v>
+        <v>0.1612600086862453</v>
       </c>
       <c r="AD2">
-        <v>0.083</v>
+        <v>0.077</v>
       </c>
       <c r="AE2">
         <v>0</v>
       </c>
       <c r="AF2">
-        <v>0.083</v>
+        <v>0.077</v>
       </c>
       <c r="AG2">
-        <v>0.083</v>
+        <v>-0.028</v>
       </c>
       <c r="AH2">
-        <v>0.08409321175278622</v>
+        <v>0.07019143117593436</v>
       </c>
       <c r="AI2">
-        <v>-0.1280864197530864</v>
+        <v>-0.1300675675675675</v>
       </c>
       <c r="AJ2">
-        <v>0.08409321175278622</v>
+        <v>-0.0282258064516129</v>
       </c>
       <c r="AK2">
-        <v>-0.1280864197530864</v>
+        <v>0.04017216642754662</v>
       </c>
       <c r="AL2">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="AM2">
-        <v>0</v>
+        <v>0.001</v>
+      </c>
+      <c r="AO2">
+        <v>-85</v>
+      </c>
+      <c r="AQ2">
+        <v>-85</v>
       </c>
     </row>
     <row r="3">
@@ -677,7 +683,7 @@
         </is>
       </c>
       <c r="K3">
-        <v>0.182</v>
+        <v>-0.105</v>
       </c>
       <c r="M3">
         <v>-0</v>
@@ -686,7 +692,7 @@
         <v>-0</v>
       </c>
       <c r="O3">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="P3">
         <v>-0</v>
@@ -695,58 +701,64 @@
         <v>-0</v>
       </c>
       <c r="R3">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="S3">
         <v>0</v>
       </c>
       <c r="U3">
-        <v>0</v>
+        <v>0.105</v>
       </c>
       <c r="V3">
-        <v>0</v>
+        <v>0.1029411764705882</v>
       </c>
       <c r="W3">
-        <v>-0.175</v>
+        <v>0.1436388508891929</v>
       </c>
       <c r="X3">
-        <v>0.1427779612909701</v>
+        <v>0.1647033579267986</v>
       </c>
       <c r="Y3">
-        <v>-0.3177779612909701</v>
+        <v>-0.02106450703760576</v>
       </c>
       <c r="AB3">
-        <v>0.1391722223025425</v>
+        <v>0.1612600086862453</v>
       </c>
       <c r="AD3">
-        <v>0.083</v>
+        <v>0.077</v>
       </c>
       <c r="AE3">
         <v>0</v>
       </c>
       <c r="AF3">
-        <v>0.083</v>
+        <v>0.077</v>
       </c>
       <c r="AG3">
-        <v>0.083</v>
+        <v>-0.028</v>
       </c>
       <c r="AH3">
-        <v>0.08409321175278622</v>
+        <v>0.07019143117593436</v>
       </c>
       <c r="AI3">
-        <v>-0.1280864197530864</v>
+        <v>-0.1300675675675675</v>
       </c>
       <c r="AJ3">
-        <v>0.08409321175278622</v>
+        <v>-0.0282258064516129</v>
       </c>
       <c r="AK3">
-        <v>-0.1280864197530864</v>
+        <v>0.04017216642754662</v>
       </c>
       <c r="AL3">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="AM3">
-        <v>0</v>
+        <v>0.001</v>
+      </c>
+      <c r="AO3">
+        <v>-85</v>
+      </c>
+      <c r="AQ3">
+        <v>-85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>